<commit_message>
fix(districts): adopt scheme A to re-align Mid-Levels West and Central boundaries (Castle Rd & Robinson Rd to West, Glenealy to Central)
</commit_message>
<xml_diff>
--- a/全港一手新盘空间区域与商圈归属重划表.xlsx
+++ b/全港一手新盘空间区域与商圈归属重划表.xlsx
@@ -7466,7 +7466,7 @@
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>西半山</t>
+          <t>中半山</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -7514,17 +7514,17 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>中半山</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>Mid-Levels Central</t>
+          <t>Mid-Levels West</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>FEAT-TPU-142-143</t>
+          <t>FEAT-S-H11</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -7582,17 +7582,17 @@
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>中半山</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>Mid-Levels Central</t>
+          <t>Mid-Levels West</t>
         </is>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>FEAT-TPU-142-143</t>
+          <t>FEAT-S-H11</t>
         </is>
       </c>
       <c r="G101" s="6" t="inlineStr">
@@ -7658,17 +7658,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>中半山</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>Mid-Levels Central</t>
+          <t>Mid-Levels West</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>FEAT-TPU-142-143</t>
+          <t>FEAT-S-H11</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -7734,17 +7734,17 @@
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>中半山</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>Mid-Levels Central</t>
+          <t>Mid-Levels West</t>
         </is>
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>FEAT-TPU-142-143</t>
+          <t>FEAT-S-H11</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
@@ -7822,7 +7822,7 @@
       </c>
       <c r="H104" s="4" t="inlineStr">
         <is>
-          <t>西半山</t>
+          <t>中半山</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -7878,17 +7878,17 @@
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>中半山</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>Mid-Levels Central</t>
+          <t>Mid-Levels West</t>
         </is>
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>FEAT-TPU-142-143</t>
+          <t>FEAT-S-H11</t>
         </is>
       </c>
       <c r="G105" s="6" t="inlineStr">
@@ -8854,17 +8854,17 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>西营盘及石塘咀 / 上环</t>
+          <t>中半山</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t>Statutory Scheme (S/H3/34)</t>
+          <t>Mid-Levels Central</t>
         </is>
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
-          <t>OZP-S-H3-34</t>
+          <t>FEAT-TPU-142-143</t>
         </is>
       </c>
       <c r="G119" s="6" t="inlineStr">

</xml_diff>